<commit_message>
fix: CORS open policy, GC cleanup in eval loop, remove branding from UI footer
</commit_message>
<xml_diff>
--- a/reports/evaluation_report.xlsx
+++ b/reports/evaluation_report.xlsx
@@ -494,7 +494,7 @@
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>25</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
@@ -564,7 +564,7 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="7">
@@ -579,7 +579,7 @@
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.76</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="8">
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>0.88</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="9">
@@ -609,7 +609,7 @@
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -624,7 +624,7 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>0.541017316017316</v>
+        <v>0.5314285714285714</v>
       </c>
     </row>
     <row r="11">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.68</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="12">
@@ -699,7 +699,7 @@
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>0.72</v>
+        <v>0.5999999999999999</v>
       </c>
     </row>
     <row r="16">
@@ -714,7 +714,7 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>0.52</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="17">
@@ -729,7 +729,7 @@
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>0.5416666666666666</v>
+        <v>0.7777777777777778</v>
       </c>
     </row>
     <row r="18">
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="C19" s="6" t="n">
-        <v>0.1946666666666667</v>
+        <v>0.8766666666666666</v>
       </c>
     </row>
     <row r="20">
@@ -774,7 +774,7 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>0.2027777777777778</v>
+        <v>0.8629629629629629</v>
       </c>
     </row>
     <row r="21">
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="C21" s="6" t="n">
-        <v>0.04</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -819,7 +819,7 @@
         </is>
       </c>
       <c r="C23" s="6" t="n">
-        <v>0.04166666666666666</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -833,15 +833,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -897,19 +897,19 @@
         </is>
       </c>
       <c r="B4" s="7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C4" s="4" t="n">
         <v>1</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>0.9166666666666666</v>
+        <v>0.8666666666666668</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>0.25</v>
+        <v>1.1</v>
       </c>
       <c r="G4" s="4" t="n">
         <v>0</v>
@@ -922,19 +922,19 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.7272727272727273</v>
+        <v>0.75</v>
       </c>
       <c r="D5" s="10" t="n">
-        <v>0.606060606060606</v>
+        <v>0.4166666666666666</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.6363636363636364</v>
+        <v>0.75</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.09393939393939393</v>
+        <v>0.5666666666666667</v>
       </c>
       <c r="G5" s="6" t="n">
         <v>0</v>
@@ -943,50 +943,25 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Multi_hop</t>
+          <t>Unanswerable</t>
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="E6" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>0.3666666666666666</v>
+        <v>1</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Unanswerable</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1006,10 +981,10 @@
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -1065,19 +1040,19 @@
         </is>
       </c>
       <c r="B4" s="7" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>0.9</v>
+        <v>0.75</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>0.8333333333333333</v>
+        <v>0.5833333333333333</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>0.1666666666666667</v>
+        <v>1.025</v>
       </c>
       <c r="G4" s="4" t="n">
         <v>0</v>
@@ -1090,22 +1065,22 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="D5" s="10" t="n">
         <v>0.6666666666666666</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.275</v>
+        <v>1</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.125</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -1115,19 +1090,19 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>0.8333333333333334</v>
+        <v>1</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>0.7222222222222223</v>
+        <v>0.7777777777777778</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>0.6666666666666666</v>
+        <v>1</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>0.1666666666666667</v>
+        <v>0.5555555555555555</v>
       </c>
       <c r="G6" s="4" t="n">
         <v>0</v>
@@ -1152,7 +1127,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" s="6" t="n">
         <v>0</v>
@@ -1169,15 +1144,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="29" customWidth="1" min="8" max="8"/>
   </cols>
@@ -1249,22 +1224,22 @@
         </is>
       </c>
       <c r="D4" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>interpretive</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="n">
         <v>0.75</v>
       </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>interpretive</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>0.6363636363636364</v>
-      </c>
       <c r="G4" s="8" t="n">
-        <v>0.2473721448347073</v>
+        <v>0.1199023331949856</v>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Small Effect (0.2 - 0.5)</t>
+          <t>Negligible (&lt; 0.2)</t>
         </is>
       </c>
     </row>
@@ -1293,158 +1268,14 @@
         </is>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.7272727272727273</v>
+        <v>0.75</v>
       </c>
       <c r="G5" s="10" t="n">
-        <v>1.098934489515254</v>
+        <v>1.047197551196598</v>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
           <t>Large Effect (&gt;= 0.8)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Factual vs Multi_hop</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Citation Accuracy</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>factual</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>multi_hop</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="8" t="n">
-        <v>2.094395102393195</v>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>Large Effect (&gt;= 0.8)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Factual vs Multi_hop</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Retrieval Recall@8</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>factual</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>multi_hop</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="G7" s="10" t="n">
-        <v>0.9272952180016123</v>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>Large Effect (&gt;= 0.8)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Interpretive vs Multi_hop</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Citation Accuracy</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>interpretive</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="n">
-        <v>0.6363636363636364</v>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>multi_hop</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="8" t="n">
-        <v>1.847022957558488</v>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>Large Effect (&gt;= 0.8)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Interpretive vs Multi_hop</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Retrieval Recall@8</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>interpretive</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>0.7272727272727273</v>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>multi_hop</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="G9" s="10" t="n">
-        <v>-0.1716392715136421</v>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>Negligible (&lt; 0.2)</t>
         </is>
       </c>
     </row>
@@ -1596,14 +1427,14 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>ITW assumed the Lemelson lawsuit as part of the purchase agreement for the DeVilbiss assets [INDOPCO Inc. v. Commissioner (1992), Page 6]. 
+          <t>ITW assumed the Lemelson lawsuit as part of the purchase agreement for the DeVilbiss assets [INDOPCO Inc. v. Commissioner (1992) | Page 6]. This contingent liability formed part of the purchase price because the DeVilbiss acquisition was meant to benefit ITW into the future [INDOPCO Inc. v. Commissioner (1992) | Page 6]. 
 Sources:
-[INDOPCO Inc. v. Commissioner (1992), Page 6]</t>
+[INDOPCO Inc. v. Commissioner (1992) | Page 6]</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>INDOPCO Inc. v. Commissioner (1992) (p.6)</t>
         </is>
       </c>
       <c r="J4" s="7" t="b">
@@ -1616,10 +1447,10 @@
         <v>1</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -1650,11 +1481,10 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>IRC 61 distributions taxable event non-taxable event distinction 
-Reg 1.61-12 taxable vs non-taxable distributions 
-Commissioner v Glenshaw Glass 346 US 425 
-IRC 104 punitive damages non-taxable 
-United</t>
+          <t>IRC 61 distributions taxable event non-taxable event distinction court cases
+IRC 61 vs IRC 104 punitive damages taxation distinction
+Commissioners v Glenshaw Glass 346 US 425
+Commissioners v Schleier 515 US</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
@@ -1664,17 +1494,15 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>The court distinguished between a taxable event and a non-taxable event in the context of distributions from a company by determining whether the distribution constituted a "gain derived from capital, from labor, or from both combined" [Eisner v. Macomber, 252 U. S. 189, 207, as cited in Commissioner v. Glenshaw Glass Co. (1955), p.3]. In Eisner v. Macomber, the court held that a distribution of a corporate stock dividend did not constitute a taxable event because it did not change "only the form, not the essence," of the shareholder's capital investment [Eisner v. Macomber, 252 U. S. 189, 210, as cited in Commissioner v. Glenshaw Glass Co. (1955), p.3]. However, in the context of punitive damages, the court held that such damages constitute a taxable event because they represent an "undeniable accession to wealth, clearly realized, and over which the taxpayers have complete dominion" [Commissioner v. Glenshaw Glass Co. (1955), p.3]. This distinction implies that punitive damages are subject to taxation because they are not considered a return of capital, but rather a gain or profit that is within the scope of § 22 (a) [Helvering v. Bruun (1940), p.4]. 
-Sources: 
-[Commissioner v. Glenshaw Glass Co. (1955), p.3] 
-[Helvering v. Bruun (1940), p.4] 
-[Eisner v. Macomber, 252 U. S. 189, 207, as cited in Commissioner v. Glenshaw Glass Co. (1955), p.3] 
-[Eisner v. Macomber, 252 U. S. 189, 210, as cited in Commissioner v. Glenshaw Glass Co. (1955), p.3]</t>
+          <t>The court distinguished between a taxable event and a non-taxable event in the context of distributions from a company by considering whether the distribution constituted a "realized gain" to the shareholder, or merely a change in the form of the shareholder's capital investment [Helvering v. Bruun, p.3]. In Eisner v. Macomber, the court held that a distribution of a corporate stock dividend did not constitute a taxable event because it did not result in a gain to the shareholder, but rather only a change in the form of their capital investment [Eisner v. Macomber, as cited in Commissioner v. Glenshaw Glass Co. (1955) | Page 3]. In contrast, the court found that punitive damages, which are a form of "undeniable accessions to wealth" [Commissioner v. Glenshaw Glass Co. (1955) | Page 3], are taxable because they constitute a realized gain to the recipient, and are not merely a return of capital [Helvering v. Bruun, p.3]. This distinction has implications for the taxation of punitive damages, as it suggests that such damages are subject to taxation as ordinary income, rather than being exempt from taxation as non-taxable gifts or returns of capital [Commissioner v. Glenshaw Glass Co. (1955) | Page 3].
+Sources:
+[Commissioner v. Glenshaw Glass Co. (1955) | Page 3]
+[Helvering v. Bruun, p.3]</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Commissioner v. Glenshaw Glass Co. (1955) (p.3), Helvering v. Bruun (1940) (p.4)</t>
+          <t>Helvering v. Bruun (1940) (p.3), Commissioner v. Glenshaw Glass Co. (1955) (p.3)</t>
         </is>
       </c>
       <c r="J5" s="9" t="b">
@@ -1687,10 +1515,10 @@
         <v>0.3333333333333333</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -1721,7 +1549,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>IRC 165 Subsec h1 Pub L 92-336 substitution made</t>
+          <t>IRC 165 Subsec h1 Pub L 92-336 substitution</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -1731,14 +1559,12 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Pub. L. 92–336 substituted provisions relating to losses attributable to a disaster which occurs during the period after the close of the taxable year and on or before the last day of the 6th calendar month beginning after the close of the taxable year, for provisions relating to losses attributable to a disaster which occurs during the period following the close of the taxable year and on or before the time prescribed by law for filing the income tax return for the taxable year, determined without regard to any extension of time [IRC Section 165 - Losses, p.6]. 
-Sources: 
-[IRC Section 165 - Losses, p.6]</t>
+          <t>Pub. L. 92–336 substituted provisions relating to losses attributable to a disaster which occurs during the period after the close of the taxable year and on or before the last day of the 6th calendar month beginning after the close of the taxable year, for provisions relating to losses attributable to a disaster which occurs during the period following the close of the taxable year and on or before the time prescribed by law for filing the income tax return for the taxable year, determined without regard to any extension of time [CONTEXT 1] IRC Section 165 - Losses | Page 6 | IRC §165, p.6].</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>IRC Section 165 - Losses (p.6)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J6" s="7" t="b">
@@ -1751,10 +1577,10 @@
         <v>1</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -1795,15 +1621,17 @@
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Section 220 is referenced in the phrase 'The deduction allowed by section 220' in IRC §62 [IRC Section 62 - Adjusted Gross Income Defined | Page 6, p.450] and [IRC Section 62 - Adjusted Gross Income Defined | Page 5, p. no page number]. 
-Sources: 
-[IRC Section 62 - Adjusted Gross Income Defined | Page 6, p.450] 
-[IRC Section 62 - Adjusted Gross Income Defined | Page 5]</t>
+          <t>The section referenced in the phrase 'The deduction allowed by section 220' in IRC §62 is Section 220, which relates to retirement savings for certain married individuals [IRC Section 62 - Adjusted Gross Income Defined | Page 6, p.1] and also referred to in [IRC Section 62 - Adjusted Gross Income Defined | Page 5, p.1] and [IRC Section 62 - Adjusted Gross Income Defined | Page 3, p.1] and [IRC Section 62 - Adjusted Gross Income Defined | Page 2, p.1].
+Sources:
+[IRC Section 62 - Adjusted Gross Income Defined | Page 6, p.1]
+[IRC Section 62 - Adjusted Gross Income Defined | Page 5, p.1]
+[IRC Section 62 - Adjusted Gross Income Defined | Page 3, p.1]
+[IRC Section 62 - Adjusted Gross Income Defined | Page 2, p.1]</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>IRC Section 62 - Adjusted Gross Income Defined | Page 6 (p.1), IRC Section 62 - Adjusted Gross Income Defined (p.6), IRC Section 62 - Adjusted Gross Income Defined (p.5), IRC Section 62 - Adjusted Gross Income Defined (p.3), IRC Section 62 - Adjusted Gross Income Defined (p.2)</t>
         </is>
       </c>
       <c r="J7" s="9" t="b">
@@ -1816,10 +1644,10 @@
         <v>0.3333333333333333</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -1860,14 +1688,15 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>The deadline for filing an amended tax return for IRA contributions made in 2026 is the regular due date for amending a return [IRS Publication 590A - IRA Contributions, p.31]. 
-Sources: 
-[IRS Publication 590A - IRA Contributions, p.31]</t>
+          <t>The deadline for filing an amended tax return for IRA contributions made in 2026 is the regular due date for amending a return [IRS Publication 590A - IRA Contributions | Page 31]. Additionally, if you miss the deadline for recharacterizing a contribution, you can still recharacterize it within 6 months from the due date of your return, excluding extensions [IRS Publication 590A - IRA Contributions | Page 30]. 
+Sources:
+[IRS Publication 590A - IRA Contributions | Page 30]
+[IRS Publication 590A - IRA Contributions | Page 31]</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>IRS Publication 590A - IRA Contributions (p.31)</t>
+          <t>IRS Publication 590A - IRA Contributions (p.31), IRS Publication 590A - IRA Contributions (p.30)</t>
         </is>
       </c>
       <c r="J8" s="7" t="b">
@@ -1883,7 +1712,7 @@
         <v>0</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -1924,11 +1753,11 @@
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>$25,000 [IRC Section 7201 - Tax Evasion | Page 1 | IRC §7201, p.3850] and [IRC Section 7201 - Tax Evasion | Page 1 | IRC §7201, p.1] and [IRC Section 7203, p.3850]
+          <t>The maximum fine for an individual found guilty of a misdemeanor under IRC §7203, not IRC §7201, is $25,000 [IRC Section 7201 - Tax Evasion | Page 1 | IRC §7201, p.1] [IRC Section 7203, p.1]. However, for a felony under IRC §7201, the maximum fine is $100,000 for an individual [IRC Section 7201 - Tax Evasion | Page 1 | IRC §7201, p.1]. 
 Sources:
-[IRC Section 7201 - Tax Evasion | Page 1 | IRC §7201, p.3850]
 [IRC Section 7201 - Tax Evasion | Page 1 | IRC §7201, p.1]
-[IRC Section 7203, p.3850]</t>
+[CONTEXT 1] IRC Section 7201 - Tax Evasion | Page 1 | IRC §7201 
+[CONTEXT 3] IRC Section 7201 - Tax Evasion | Page 1 | IRC §7201</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
@@ -1949,7 +1778,7 @@
         <v>1</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="10">
@@ -1990,15 +1819,14 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>The maximum amount that can be excluded from an employee's gross income for the adoption of a child with special needs for taxable years beginning in 2022 is $14,890 [Jct Report: 05 Corps, p.15] and [Jct Report: 05 Corps, p.9].
+          <t>The maximum amount that can be excluded from an employee's gross income for the adoption of a child with special needs for taxable years beginning in 2022 is $14,890 [Jct Report: 05 Corps | Page 15]. 
 Sources:
-[Jct Report: 05 Corps, p.15]
-[Jct Report: 05 Corps, p.9]</t>
+[Jct Report: 05 Corps | Page 15]</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Jct Report: 05 Corps (p.15), Jct Report: 05 Corps (p.9)</t>
+          <t>Jct Report: 05 Corps (p.15)</t>
         </is>
       </c>
       <c r="J10" s="7" t="b">
@@ -2014,7 +1842,7 @@
         <v>1</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -2055,19 +1883,17 @@
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>The context of IRC Section 408 implies that the legislative intent behind the creation of Individual Retirement Accounts (IRAs) is to encourage private savings for retirement, as evident from the various provisions and limitations on contributions to IRAs [Crs Report: 07 Ira, p.2] and [Crs Report: 03 Charitable, p.2]. The creation of Roth IRAs, in particular, is intended to provide an alternative to traditional IRAs, with after-tax contributions and tax-free distributions [IRS Publication 590A - IRA Contributions, p.39]. The legislative intent is also reflected in the rules and regulations governing IRAs, such as the eligibility requirements, contribution limits, and distribution rules [IRS Publication 590A - IRA Contributions, p.1] and [Gao Report: 04 Penalties, p.3]. Furthermore, the context suggests that the legislative intent is to provide a means for individuals to save for retirement, with the goal of reducing reliance on other sources of support, such as Social Security and employer pensions [Gao Report: 04 Penalties, p.1].
+          <t>The context of IRC Section 408 implies that the legislative intent behind the creation of Individual Retirement Accounts (IRAs) is to encourage private savings for retirement [Crs Report: 07 Ira, Page 2]. This is further supported by the fact that IRAs have been one of the government’s primary programs aimed at encouraging private savings since the early 1980s [Gao Report: 04 Penalties, Page 3]. The creation of Roth IRAs, which allow for after-tax contributions, also suggests an intent to provide individuals with more options for saving for retirement [Gao Report: 04 Penalties, Page 3]. Additionally, the rules and regulations surrounding IRAs, such as the contribution limits and eligibility requirements, imply an intent to ensure that these accounts are used for their intended purpose of providing retirement savings [IRS Publication 590A - IRA Contributions, Page 1]. The ability to make nondeductible contributions to a Roth IRA, regardless of age, also suggests an intent to encourage retirement savings [IRS Publication 590A - IRA Contributions, Page 39].
 Sources:
-[Crs Report: 07 Ira, p.2]
-[Crs Report: 03 Charitable, p.2]
-[IRS Publication 590A - IRA Contributions, p.1]
-[IRS Publication 590A - IRA Contributions, p.39]
-[Gao Report: 04 Penalties, p.1]
-[Gao Report: 04 Penalties, p.3]</t>
+[Crs Report: 07 Ira, Page 2]
+[Gao Report: 04 Penalties, Page 3]
+[IRS Publication 590A - IRA Contributions, Page 1]
+[IRS Publication 590A - IRA Contributions, Page 39]</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Crs Report: 07 Ira (p.2), Crs Report: 03 Charitable (p.2), IRS Publication 590A - IRA Contributions (p.39), IRS Publication 590A - IRA Contributions (p.1), Gao Report: 04 Penalties (p.3)</t>
+          <t>Crs Report: 07 Ira (p.2), Gao Report: 04 Penalties (p.3), IRS Publication 590A - IRA Contributions (p.1), IRS Publication 590A - IRA Contributions (p.39)</t>
         </is>
       </c>
       <c r="J11" s="9" t="b">
@@ -2083,7 +1909,7 @@
         <v>0</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="12">
@@ -2115,7 +1941,10 @@
       <c r="F12" s="3" t="inlineStr">
         <is>
           <t>IRC 1272 OID accrual subsequent periods formula values 
-issue price adjusted OID accrual period original issue discount accrual period</t>
+issue price adjusted OID accrual period end balance 
+adjusted issue price adjusted OID accrual period end balance 
+adjusted issue price adjusted OID accrual period end balance 
+adjusted issue price adjusted OID accr</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -2125,16 +1954,16 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>The calculation of daily Original Issue Discount (OID) for subsequent accrual periods changes in that the adjusted issue price at the beginning of each period is used in the formula instead of the issue price [Jct Report: 02 Expenditures, p.13] and [Jct Report: 02 Expenditures, p.11]. The adjusted issue price is the sum of the issue price and all the OID includible in income before that accrual period minus any payment previously made on the debt instrument, other than a payment of qualified stated interest [Jct Report: 02 Expenditures, p.3]. 
+          <t>The calculation of daily Original Issue Discount (OID) for subsequent accrual periods is figured the same way as the initial accrual period, except the adjusted issue price at the beginning of each period is used in the formula instead of the issue price [Jct Report: 02 Expenditures | Page 13]. The adjusted issue price is the sum of the issue price and all the OID includible in income before that accrual period minus any payment previously made on the debt instrument, other than a payment of qualified stated interest [Jct Report: 02 Expenditures | Page 3]. The daily OID for subsequent accrual periods is figured using the formula: (adjusted issue price x yield to maturity) / number of days in accrual period - qualified stated interest / number of days in accrual period [Jct Report: 02 Expenditures | Page 11]. 
 Sources:
-[Jct Report: 02 Expenditures, p.13] 
-[Jct Report: 02 Expenditures, p.11] 
-[Jct Report: 02 Expenditures, p.3]</t>
+[Jct Report: 02 Expenditures | Page 3]
+[Jct Report: 02 Expenditures | Page 11]
+[Jct Report: 02 Expenditures | Page 13]</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Jct Report: 02 Expenditures (p.13), Jct Report: 02 Expenditures (p.11), Jct Report: 02 Expenditures (p.3)</t>
+          <t>Jct Report: 02 Expenditures (p.13), Jct Report: 02 Expenditures (p.3), Jct Report: 02 Expenditures (p.11)</t>
         </is>
       </c>
       <c r="J12" s="7" t="b">
@@ -2150,7 +1979,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
     </row>
     <row r="13">
@@ -2191,12 +2020,11 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>The safe harbor rules under § 1.148-5(e)(2)(iii)(B)(1) of the Income Tax Regulations determine the reasonableness of a broker's commission for the acquisition of a guaranteed investment contract or investments purchased for a yield restricted defeasance escrow by considering two conditions: (1) the amount of the fee that the issuer treats as a qualified administrative cost does not exceed the lesser of (A) a specified amount, and (B) 0.2 percent of the computational base or, if more, a specified amount; and (2) for any issue, the issuer does not treat more than a specified amount in brokers’ commissions or similar fees as qualified administrative costs for all guaranteed investment contracts and investments for yield restricted defeasance escrows purchased with gross proceeds of the issue [Jct Report: 04 Retirement, p.15], [Jct Report: 05 Corps, p.16], [Tax Foundation: 05 1031, p.14]. 
-Specifically, for calendar year 2023, the amount of the fee is reasonable if it does not exceed the lesser of (A) $46,000, and (B) 0.2 percent of the computational base or, if more, $5,000; and the issuer does not treat more than $130,000 in brokers’ commissions or similar fees as qualified administrative costs [Jct Report: 04 Retirement, p.15]. For calendar year 2022, the amount of the fee is reasonable if it does not exceed the lesser of (A) $43,000, and (B) 0.2 percent of the computational base or, if more, $4,000; and the issuer does not treat more than $122,000 in brokers’ commissions or similar fees as qualified administrative costs [Jct Report: 05 Corps, p.16]. For calendar year 2024, the amount of the fee is reasonable if it does not exceed the lesser of (A) $49,000, and (B) 0.2 percent of the computational base or, if more, $5,000; and the issuer does not treat more than $138,000 in brokers’ commissions or similar fees as qualified administrative costs [Tax Foundation: 05 1031, p.14]. 
-Sources: 
-[Jct Report: 04 Retirement, p.15] 
-[Jct Report: 05 Corps, p.16] 
-[Tax Foundation: 05 1031, p.14]</t>
+          <t>The safe harbor rules under § 1.148-5(e)(2)(iii)(B)(1) of the Income Tax Regulations determine the reasonableness of a broker's commission for the acquisition of a guaranteed investment contract or investments purchased for a yield restricted defeasance escrow if (1) the amount of the fee that the issuer treats as a qualified administrative cost does not exceed the lesser of (A) $46,000, and (B) 0.2 percent of the computational base or, if more, $5,000; and (2) for any issue, the issuer does not treat more than $130,000 in brokers’ commissions or similar fees as qualified administrative costs for all guaranteed investment contracts and investments for yield restricted defeasance escrows purchased with gross proceeds of the issue [Jct Report: 04 Retirement | Page 15]. For calendar year 2022, the amounts are $43,000 and $122,000 [Jct Report: 05 Corps | Page 16]. For calendar year 2024, the amounts are $49,000 and $138,000 [Tax Foundation: 05 1031 | Page 14]. 
+Sources:
+[Jct Report: 04 Retirement | Page 15]
+[Jct Report: 05 Corps | Page 16]
+[Tax Foundation: 05 1031 | Page 14]</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
@@ -2246,11 +2074,7 @@
           <t>How does the legislative intent, as reflected in the amendments to section 6662, influence the interpretation of the accuracy-related penalty under the Internal Revenue Code of 1986?</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>IRC 6662 accuracy-related penalty legislative intent amendment influence interpretation</t>
-        </is>
-      </c>
+      <c r="F14" s="3" t="inlineStr"/>
       <c r="G14" s="3" t="inlineStr">
         <is>
           <t>act_sec6662, p.4</t>
@@ -2258,29 +2082,25 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>The legislative intent, as reflected in the amendments to section 6662, influences the interpretation of the accuracy-related penalty under the Internal Revenue Code of 1986 by emphasizing the importance of accuracy and compliance with tax regulations [IRC Section 6662, p.4]. The amendments, such as those made by Pub. L. 111-152, title I, § 1409(b)(1), (2), Mar. 30, 2010, 124 Stat. 1068, 1069, demonstrate Congress's intent to strengthen the accuracy-related penalty provisions [IRC Section 6662, p.4]. Furthermore, the addition of new paragraphs, such as subsection (l) added by Pub. L. 116-260, § 212(b)(2), Dec. 27, 2020, 134 Stat. 3067, indicates a continued effort to refine and clarify the application of the accuracy-related penalty [IRC Section 6662, p.4]. The legislative history and amendments to section 6662 provide context for understanding the scope and application of the accuracy-related penalty, highlighting the need for taxpayers to accurately report their tax liabilities and comply with tax regulations [IRC Section 6662, p.1] and [Tax Foundation: 02 Capgains, p.86].
-Sources:
-[IRC Section 6662, p.4]
-[IRC Section 6662, p.1]
-[Tax Foundation: 02 Capgains, p.86]</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>IRC Section 6662 - Accuracy-Related Penalty (p.4), IRC Section 6662 - Accuracy-Related Penalty (p.1), Tax Foundation: 02 Capgains (p.86)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J14" s="7" t="b">
         <v>0</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L14" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N14" s="4" t="n">
         <v>0</v>
@@ -2312,11 +2132,7 @@
           <t>How should the amendment to IRC §121, which directs the redesignation of paragraph (9) as (10) and adds a new paragraph (9), be interpreted in light of the fact that subsection (d) did not contain a paragraph (9) at the time of the amendment?</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>IRC 121 paragraph redesignation amendment interpretation subsection d absence paragraph 9</t>
-        </is>
-      </c>
+      <c r="F15" s="5" t="inlineStr"/>
       <c r="G15" s="5" t="inlineStr">
         <is>
           <t>act_sec121, p.5</t>
@@ -2324,30 +2140,28 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>The amendment to IRC §121 should be interpreted to reflect the probable intent of Congress, and therefore, the amendment was executed by redesignating as paragraph (10) the paragraph (9) directed to be added to subsection (d) of this section by Pub. L. 107–16, § 542(c), (f)(1), applicable to estates of decedents dying after Dec. 31, 2009 [IRC Section 121 - Home Sale Exclusion, p.5]. 
-Sources: 
-[IRC Section 121 - Home Sale Exclusion, p.5]</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>IRC Section 121 - Home Sale Exclusion (p.5)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J15" s="9" t="b">
         <v>0</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L15" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -2376,11 +2190,7 @@
           <t>What did Justice Cardozo describe as a struggle to find a verbal formula to supply a ready touchstone for?</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>Justice Cardozo described a struggle to find a verbal formula to supply a ready touchstone for the concept of "substantially related"</t>
-        </is>
-      </c>
+      <c r="F16" s="3" t="inlineStr"/>
       <c r="G16" s="3" t="inlineStr">
         <is>
           <t>judgment_14_commissioner_v_duberstein, p.7</t>
@@ -2388,31 +2198,28 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>Justice Cardozo described the search for a definition of "ordinary and necessary" expenses as a struggle to find a verbal formula to supply a ready touchstone, stating that "One struggles in vain for any verbal formula that will supply a ready touchstone" [Welch v. Helvering, p.2] and also quoted in [Commissioner v. Duberstein, p.7]. 
-Sources: 
-[Commissioner v. Duberstein, p.7] 
-[Welch v. Helvering, p.2]</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Welch v. Helvering (1933) (p.2), Commissioner v. Duberstein (1960) (p.7)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J16" s="7" t="b">
         <v>0</v>
       </c>
       <c r="K16" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L16" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N16" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -2441,11 +2248,7 @@
           <t>How does the coordination with minimum tax under section 55 affect the determination of qualified business income for purposes of the deduction under subsection (a), and what implications does this have for taxpayers subject to alternative minimum taxable income?</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>IRC 199A qualified business income coordination with IRC 55 minimum tax alternative minimum taxable income implications</t>
-        </is>
-      </c>
+      <c r="F17" s="5" t="inlineStr"/>
       <c r="G17" s="5" t="inlineStr">
         <is>
           <t>act_sec199A, p.4</t>
@@ -2453,27 +2256,25 @@
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>The coordination with minimum tax under section 55 affects the determination of qualified business income for purposes of the deduction under subsection (a) by requiring that qualified business income be determined without regard to any adjustments under sections 56 through 59 for purposes of determining alternative minimum taxable income under section 55 [IRC Section 199A - Qualified Business Income Deduction, p.4]. This means that taxpayers subject to alternative minimum taxable income will have their qualified business income determined without considering certain adjustments that may be applicable for regular tax purposes, potentially affecting the amount of the deduction available to them [IRC Section 199A - Qualified Business Income Deduction, p.4]. 
-Sources: 
-[IRC Section 199A - Qualified Business Income Deduction, p.4]</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>IRC Section 199A - Qualified Business Income Deduction (p.4)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J17" s="9" t="b">
         <v>0</v>
       </c>
       <c r="K17" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L17" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>0</v>
@@ -2505,11 +2306,7 @@
           <t>What did the Supreme Court hold regarding the willfulness requirement for tax crimes in Cheek v. United States?</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>Cheek v United States IRC 7201 willfulness requirement mens rea strict scrutiny Supreme Court holding</t>
-        </is>
-      </c>
+      <c r="F18" s="3" t="inlineStr"/>
       <c r="G18" s="3" t="inlineStr">
         <is>
           <t>judgment_11_cheek_v_united_states, p.2</t>
@@ -2517,11 +2314,7 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>The Supreme Court held that a good-faith misunderstanding of the law or a good-faith belief that one is not violating the law negates willfulness, whether or not the claimed belief or misunderstanding is objectively reasonable [Cheek v. United States (1991), p. 3] and [Cheek v. United States (1991), p. 8]. The Court also stated that willfulness requires the Government to prove that the law imposed a duty on the defendant, that the defendant knew of this duty, and that he voluntarily and intentionally violated that duty [Cheek v. United States (1991), p. 6]. 
-Sources: 
-[Cheek v. United States (1991), p. 3]
-[Cheek v. United States (1991), p. 6]
-[Cheek v. United States (1991), p. 8]</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
@@ -2571,13 +2364,7 @@
           <t>What is the effective period for the amendments made by Pub. L. 115–97, and how does this relate to the substitution made by Pub. L. 105–277 in subsec. (b)(3) regarding casualty or theft losses?</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>IRC 165(h) casualty loss Pub L 115-97 effective date amendment 
-IRC 165(h) casualty loss Pub L 105-277 subsec b3 substitution 
-effective date Pub L 115-97 Tax Cuts and Jobs Act</t>
-        </is>
-      </c>
+      <c r="F19" s="5" t="inlineStr"/>
       <c r="G19" s="5" t="inlineStr">
         <is>
           <t>act_sec67, p.2</t>
@@ -2585,31 +2372,28 @@
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>The effective period for the amendments made by Pub. L. 115–97 is for taxable years beginning after December 31, 2017 [IRC Section 68 - Overall Limitation on Itemized Deductions, p.460] and [IRC Section 165 - Losses, p.6]. The substitution made by Pub. L. 105–277 in subsec. (b)(3) regarding casualty or theft losses, which substituted "for casualty or theft losses described in paragraph (2) or (3) of section 165(c) or for losses described in section 165(d)" for "for losses described in subsection (c)(3) or (d) of section 165", is related to the amendments made by Pub. L. 115–97 in the sense that both laws amend the Internal Revenue Code, but they operate in different sections and have different effective dates [IRC Section 68 - Overall Limitation on Itemized Deductions, p.460] and [IRC Section 165 - Losses, p.6]. 
-Sources: 
-[IRC Section 68 - Overall Limitation on Itemized Deductions, p.460] 
-[IRC Section 165 - Losses, p.6]</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>IRC Section 165 - Losses (p.6)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J19" s="9" t="b">
         <v>0</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L19" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M19" s="6" t="n">
         <v>0</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>0.3333333333333333</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -2638,14 +2422,7 @@
           <t>What is the appropriate balance between the jury's role and the reviewing court's duty, and how does this balance relate to the historical safeguards of the 'inviolate' right to trial by jury?</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>IRC 1861 jury function appellate review balance
-Trial by Jury Clause US Const Amend VI
-United States v Rutherford 390 US 544 1968
-Federated Radio Corp v Maltbie 363 US 428 1960</t>
-        </is>
-      </c>
+      <c r="F20" s="3" t="inlineStr"/>
       <c r="G20" s="3" t="inlineStr">
         <is>
           <t>judgment_24_hernandez_v_commissioner, p.7</t>
@@ -2653,9 +2430,7 @@
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>The appropriate balance between the jury's role as the judge of the facts and the reviewing court's duty to review criminal convictions is struck by not allowing the appellate court to "find" facts, or substitute its judgment for that of the jury; rather, when it determines that the verdict is against the great weight of the evidence presented at trial so as to be clearly wrong and unjust, it must reverse the verdict and remand for a new trial [Hernandez v. Commissioner (1989), p. 7]. This balance is essential to maintaining the historical safeguards of the "inviolate" right to trial by jury, which include the deferential standards of review applied and the prohibition against rendition of judgment upon a factual insufficiency point [Hernandez v. Commissioner (1989), p. 7]. 
-Sources: 
-[Hernandez v. Commissioner (1989), p. 7]</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
@@ -2667,10 +2442,10 @@
         <v>0</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L20" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M20" s="4" t="n">
         <v>0</v>
@@ -2705,11 +2480,7 @@
           <t>According to the provided text, what would have been the effect on the amount available for distribution if the liability of the transferor-corporation had been reduced to judgment during the taxable year in which liquidation occurred?</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
-        <is>
-          <t>IRC 312 liquidation distribution liability reduced judgment effect on amount available</t>
-        </is>
-      </c>
+      <c r="F21" s="5" t="inlineStr"/>
       <c r="G21" s="5" t="inlineStr">
         <is>
           <t>judgment_17_arrowsmith_v_commissioner, p.3</t>
@@ -2717,27 +2488,25 @@
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>The amount available for distribution would have been decreased, which would have reduced the liquidating dividends proportionately and diminished the capital gains taxes assessed against the stockholders, and probably would have also decreased the corporation's own taxable income [Arrowsmith v. Commissioner (1952), p.3]. 
-Sources: 
-[Arrowsmith v. Commissioner (1952), p.3]</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>Arrowsmith v. Commissioner (1952) (p.3)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J21" s="9" t="b">
         <v>0</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L21" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N21" s="6" t="n">
         <v>0</v>
@@ -2769,11 +2538,7 @@
           <t>How does the amendment to Subsec. (l)(1) by Pub. L. 111–152, § 1004(d)(2), affect the deductibility of amounts paid for insurance that constitutes medical care for the taxpayer, his spouse, and dependents, and what implications does this have for the interpretation of 'compensation for personal services actually rendered' in the context of IRC §162?</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>IRC 162 medical care insurance deduction amendment Pub L 111-152 1004d2 compensation personal services rendered</t>
-        </is>
-      </c>
+      <c r="F22" s="3" t="inlineStr"/>
       <c r="G22" s="3" t="inlineStr">
         <is>
           <t>act_sec162, p.11</t>
@@ -2781,30 +2546,28 @@
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>The amendment to Subsec. (l)(1) by Pub. L. 111–152, § 1004(d)(2), treats amounts paid for insurance that constitutes medical care for the taxpayer, his spouse, and dependents as "an amount for compensation for personal services actually rendered" [IRC Section 162, p.11]. This implies that such amounts are deductible as trade or business expenses under IRC §162, as they are considered compensation for personal services actually rendered [IRC Section 162, p.11]. 
-Sources:
-[IRC Section 162, p.11]</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>IRC Section 162 - Trade or Business Expenses (p.11)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J22" s="7" t="b">
         <v>0</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L22" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N22" s="4" t="n">
-        <v>0.3333333333333333</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -2833,17 +2596,7 @@
           <t>What is the relationship between the capitalization provision of § 263(a) and the depreciation allowance under § 167(a), and how does the priority-ordering directive of § 161 affect the application of these provisions?</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>IRC 263(a) capitalization provision 
-IRC 167(a) depreciation allowance 
-§ 161 priority-ordering directive 
-capital expenditures 
-tangible property 
-§ 162(a) ordinary and necessary expenses 
-§ 263(a)(1) definition</t>
-        </is>
-      </c>
+      <c r="F23" s="5" t="inlineStr"/>
       <c r="G23" s="5" t="inlineStr">
         <is>
           <t>judgment_30_commissioner_v_idaho_power, p.9</t>
@@ -2851,10 +2604,7 @@
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>The capitalization provision of § 263(a) takes precedence over the depreciation allowance under § 167(a) due to the priority-ordering directive of § 161, which requires that the deductions specified in Part VI of Subchapter B of the Income Tax Subtitle of the Code, including § 167(a), be subject to the exceptions provided in Part IX, which includes § 263(a) [Commissioner v. Idaho Power Co. (1974), p. 9]. This means that an expenditure incurred in acquiring capital assets must be capitalized, even if it might be deemed deductible under Part VI, unless an exception applies [Commissioner v. Idaho Power Co. (1974), p. 9]. The Court of Appeals erred in concluding that § 263(a) did not apply to a deduction allowed by the Code, such as depreciation of property used in a trade or business, and overlooked the contrary direction of § 161 [Commissioner v. Idaho Power Co. (1974), p. 9]. 
-Sources: 
-[Commissioner v. Idaho Power Co. (1974), p. 9] 
-[Commissioner v. Idaho Power Co. (1974), p. 17]</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr">
@@ -2866,10 +2616,10 @@
         <v>0</v>
       </c>
       <c r="K23" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L23" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M23" s="6" t="n">
         <v>0</v>
@@ -2904,11 +2654,7 @@
           <t>What was the substituted amount for '65' in Subsec. (f)(2)(A) by Pub. L. 105–178, § 9010(c)(1)?</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>26 USC 9010(c)(1) Pub L 105–178 Subsec f2A substituted amount 65</t>
-        </is>
-      </c>
+      <c r="F24" s="3" t="inlineStr"/>
       <c r="G24" s="3" t="inlineStr">
         <is>
           <t>act_sec132, p.6</t>
@@ -2916,25 +2662,25 @@
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>The substituted amount for '65' in Subsec. (f)(2)(A) by Pub. L. 105–178, § 9010(c)(1) was '$100' [IRC Section 132 - Fringe Benefits, p.6].</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>IRC Section 132 - Fringe Benefits (p.6)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J24" s="7" t="b">
         <v>0</v>
       </c>
       <c r="K24" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L24" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M24" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N24" s="4" t="n">
         <v>0</v>
@@ -2966,12 +2712,7 @@
           <t>What inference can be drawn from the defendants' decision not to provide a correct license, and how does this relate to the meaning of the letter mentioning Tom's arrival and the plan to go south tomorrow?</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>I'm a legal search query optimizer for US tax law. I can help you with that. However, the provided question seems to be more related to a general legal or contractual issue rather than US tax law. 
-That being said, here's a</t>
-        </is>
-      </c>
+      <c r="F25" s="5" t="inlineStr"/>
       <c r="G25" s="5" t="inlineStr">
         <is>
           <t>judgment_22_united_states_v_gilmore, p.8</t>
@@ -2979,7 +2720,7 @@
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>INSUFFICIENT_CONTEXT: The provided documents do not contain enough information to answer this question.</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr">
@@ -2988,7 +2729,7 @@
         </is>
       </c>
       <c r="J25" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K25" s="6" t="n">
         <v>0</v>
@@ -3000,7 +2741,7 @@
         <v>0</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -3029,11 +2770,7 @@
           <t>How does the exception to the partial interest rule for 'qualified conservation contributions' reconcile the general disallowance of deductions for contributions of less than the taxpayer's entire interest in property?</t>
         </is>
       </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>IRC 170(h) qualified conservation contribution partial interest rule exception</t>
-        </is>
-      </c>
+      <c r="F26" s="3" t="inlineStr"/>
       <c r="G26" s="3" t="inlineStr">
         <is>
           <t>pov_tf_02_capgains, p.62</t>
@@ -3041,29 +2778,25 @@
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>The exception to the partial interest rule for 'qualified conservation contributions' reconciles the general disallowance of deductions for contributions of less than the taxpayer's entire interest in property by allowing a deduction for the fair market value of the donated easement, determined as of the time of the contribution, if the easement is a qualified real property interest contributed to a qualified organization exclusively for conservation purposes [Tax Foundation: 02 Capgains, p.62] and [IRC Section 170, p.10]. This exception is specifically stated in IRC Section 170, which provides that the general rule disallowing deductions for partial interests does not apply to a qualified conservation contribution [IRC Section 170, p.10]. Additionally, IRS Publication 526 explains that a qualified conservation contribution is an exception to the partial interest rule, allowing a deduction for the contribution of a partial interest in property [IRS Publication 526, p.13]. 
-Sources: 
-[Tax Foundation: 02 Capgains, p.62] 
-[IRC Section 170, p.10] 
-[IRS Publication 526, p.13]</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>Tax Foundation: 02 Capgains (p.62), IRC Section 170 - Charitable Contributions (p.10), IRS Publication 526 - Charitable Contributions (p.13)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J26" s="7" t="b">
         <v>0</v>
       </c>
       <c r="K26" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L26" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M26" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N26" s="4" t="n">
         <v>0</v>
@@ -3095,11 +2828,7 @@
           <t>What are the conditions under which a taxpayer can revoke a § 168(k)(7) election, and how does the revocation apply to depreciable property placed in service during the same taxable year?</t>
         </is>
       </c>
-      <c r="F27" s="5" t="inlineStr">
-        <is>
-          <t>IRC 168(k)(7) election revocation conditions depreciable property placed service taxable year same year placed in service</t>
-        </is>
-      </c>
+      <c r="F27" s="5" t="inlineStr"/>
       <c r="G27" s="5" t="inlineStr">
         <is>
           <t>pov_crs_09_depreciation, p.15</t>
@@ -3107,9 +2836,7 @@
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>A taxpayer can revoke a § 168(k)(7) election if the taxpayer placed in service depreciable property during its 2018, 2019, or 2020 taxable year, made a § 168(k)(7) election on its timely filed original Federal income tax return or Form 1065 for the placed-in-service year of such depreciable property, and such return was filed on or before April 17, 2020, or made a § 168(k)(7) election in accordance with section 4 or 5 of Rev. Proc. 2019-33, respectively, for the placed-in-service year of such depreciable property on or before April 17, 2020 [Crs Report: 09 Depreciation | Page 15]. The revocation applies to all property included in the class of property and placed in service during the same taxable year [Crs Report: 09 Depreciation | Page 15]. 
-Sources: 
-[Crs Report: 09 Depreciation | Page 15]</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
@@ -3121,16 +2848,16 @@
         <v>0</v>
       </c>
       <c r="K27" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L27" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M27" s="6" t="n">
         <v>0</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -3159,11 +2886,7 @@
           <t>According to GAO analysis, what factors affect taxpayer compliance with IRS penalty provisions?</t>
         </is>
       </c>
-      <c r="F28" s="3" t="inlineStr">
-        <is>
-          <t>IRC 6651 failure to pay penalty factors affecting taxpayer compliance GAO analysis IRS penalty provisions taxpayer behavior</t>
-        </is>
-      </c>
+      <c r="F28" s="3" t="inlineStr"/>
       <c r="G28" s="3" t="inlineStr">
         <is>
           <t>pov_gao_04_penalties, p.1</t>
@@ -3171,15 +2894,12 @@
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>Taxpayer compliance with IRS penalty provisions is affected by factors such as the perception that evasion is widespread, which reduces the perceived probability of detection [Gao Report: 03 Retirement, p.26], and the behavior of other taxpayers, as the probability that a particular taxpayer is audited is lower when more taxpayers misreport their income [Gao Report: 03 Retirement, p.26]. Additionally, the use of tax practitioners can also impact compliance, as they can reduce a taxpayer's filing costs and costs associated with an audit [Gao Report: 03 Retirement, p.26]. The availability of information reporting is another factor that can improve compliance [Gao Report: 03 Retirement, p.21]. 
-Sources: 
-[Gao Report: 03 Retirement, p.26] 
-[Gao Report: 03 Retirement, p.21]</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>Gao Report: 03 Retirement (p.26), Gao Report: 03 Retirement (p.21)</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J28" s="7" t="b">
@@ -3232,7 +2952,7 @@
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
@@ -3290,7 +3010,7 @@
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
@@ -3348,7 +3068,7 @@
       </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr">
@@ -3406,7 +3126,7 @@
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
@@ -3464,7 +3184,7 @@
       </c>
       <c r="H33" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr">
@@ -3522,7 +3242,7 @@
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
@@ -3580,7 +3300,7 @@
       </c>
       <c r="H35" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I35" s="5" t="inlineStr">
@@ -3638,7 +3358,7 @@
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
@@ -3696,7 +3416,7 @@
       </c>
       <c r="H37" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I37" s="5" t="inlineStr">
@@ -3754,7 +3474,7 @@
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
@@ -3812,7 +3532,7 @@
       </c>
       <c r="H39" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I39" s="5" t="inlineStr">
@@ -3870,7 +3590,7 @@
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
@@ -3928,7 +3648,7 @@
       </c>
       <c r="H41" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I41" s="5" t="inlineStr">
@@ -3986,7 +3706,7 @@
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I42" s="3" t="inlineStr">
@@ -4044,7 +3764,7 @@
       </c>
       <c r="H43" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I43" s="5" t="inlineStr">
@@ -4102,7 +3822,7 @@
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
@@ -4160,7 +3880,7 @@
       </c>
       <c r="H45" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I45" s="5" t="inlineStr">
@@ -4218,7 +3938,7 @@
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
@@ -4276,7 +3996,7 @@
       </c>
       <c r="H47" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I47" s="5" t="inlineStr">
@@ -4334,7 +4054,7 @@
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I48" s="3" t="inlineStr">
@@ -4392,7 +4112,7 @@
       </c>
       <c r="H49" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I49" s="5" t="inlineStr">
@@ -4450,7 +4170,7 @@
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I50" s="3" t="inlineStr">
@@ -4508,7 +4228,7 @@
       </c>
       <c r="H51" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I51" s="5" t="inlineStr">
@@ -4566,7 +4286,7 @@
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I52" s="3" t="inlineStr">
@@ -4624,7 +4344,7 @@
       </c>
       <c r="H53" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I53" s="5" t="inlineStr">
@@ -4682,7 +4402,7 @@
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I54" s="3" t="inlineStr">
@@ -4740,7 +4460,7 @@
       </c>
       <c r="H55" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I55" s="5" t="inlineStr">
@@ -4798,7 +4518,7 @@
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I56" s="3" t="inlineStr">
@@ -4856,7 +4576,7 @@
       </c>
       <c r="H57" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I57" s="5" t="inlineStr">
@@ -4914,7 +4634,7 @@
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I58" s="3" t="inlineStr">
@@ -4972,7 +4692,7 @@
       </c>
       <c r="H59" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I59" s="5" t="inlineStr">
@@ -5030,7 +4750,7 @@
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I60" s="3" t="inlineStr">
@@ -5088,7 +4808,7 @@
       </c>
       <c r="H61" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I61" s="5" t="inlineStr">
@@ -5146,7 +4866,7 @@
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I62" s="3" t="inlineStr">
@@ -5204,7 +4924,7 @@
       </c>
       <c r="H63" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I63" s="5" t="inlineStr">
@@ -5262,7 +4982,7 @@
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I64" s="3" t="inlineStr">
@@ -5320,7 +5040,7 @@
       </c>
       <c r="H65" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I65" s="5" t="inlineStr">
@@ -5378,7 +5098,7 @@
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I66" s="3" t="inlineStr">
@@ -5436,7 +5156,7 @@
       </c>
       <c r="H67" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I67" s="5" t="inlineStr">
@@ -5494,7 +5214,7 @@
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I68" s="3" t="inlineStr">
@@ -5552,7 +5272,7 @@
       </c>
       <c r="H69" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I69" s="5" t="inlineStr">
@@ -5610,7 +5330,7 @@
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I70" s="3" t="inlineStr">
@@ -5668,7 +5388,7 @@
       </c>
       <c r="H71" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I71" s="5" t="inlineStr">
@@ -5726,7 +5446,7 @@
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I72" s="3" t="inlineStr">
@@ -5784,7 +5504,7 @@
       </c>
       <c r="H73" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I73" s="5" t="inlineStr">
@@ -5842,7 +5562,7 @@
       </c>
       <c r="H74" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I74" s="3" t="inlineStr">
@@ -5900,7 +5620,7 @@
       </c>
       <c r="H75" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I75" s="5" t="inlineStr">
@@ -5958,7 +5678,7 @@
       </c>
       <c r="H76" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I76" s="3" t="inlineStr">
@@ -6016,7 +5736,7 @@
       </c>
       <c r="H77" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I77" s="5" t="inlineStr">
@@ -6074,7 +5794,7 @@
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I78" s="3" t="inlineStr">
@@ -6132,7 +5852,7 @@
       </c>
       <c r="H79" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I79" s="5" t="inlineStr">
@@ -6190,7 +5910,7 @@
       </c>
       <c r="H80" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I80" s="3" t="inlineStr">
@@ -6248,7 +5968,7 @@
       </c>
       <c r="H81" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I81" s="5" t="inlineStr">
@@ -6306,7 +6026,7 @@
       </c>
       <c r="H82" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I82" s="3" t="inlineStr">
@@ -6364,7 +6084,7 @@
       </c>
       <c r="H83" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I83" s="5" t="inlineStr">
@@ -6422,7 +6142,7 @@
       </c>
       <c r="H84" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I84" s="3" t="inlineStr">
@@ -6480,7 +6200,7 @@
       </c>
       <c r="H85" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I85" s="5" t="inlineStr">
@@ -6538,7 +6258,7 @@
       </c>
       <c r="H86" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I86" s="3" t="inlineStr">
@@ -6596,7 +6316,7 @@
       </c>
       <c r="H87" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I87" s="5" t="inlineStr">
@@ -6654,7 +6374,7 @@
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I88" s="3" t="inlineStr">
@@ -6712,7 +6432,7 @@
       </c>
       <c r="H89" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I89" s="5" t="inlineStr">
@@ -6770,7 +6490,7 @@
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I90" s="3" t="inlineStr">
@@ -6828,7 +6548,7 @@
       </c>
       <c r="H91" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I91" s="5" t="inlineStr">
@@ -6886,7 +6606,7 @@
       </c>
       <c r="H92" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I92" s="3" t="inlineStr">
@@ -6944,7 +6664,7 @@
       </c>
       <c r="H93" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I93" s="5" t="inlineStr">
@@ -7002,7 +6722,7 @@
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I94" s="3" t="inlineStr">
@@ -7060,7 +6780,7 @@
       </c>
       <c r="H95" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I95" s="5" t="inlineStr">
@@ -7118,7 +6838,7 @@
       </c>
       <c r="H96" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I96" s="3" t="inlineStr">
@@ -7176,7 +6896,7 @@
       </c>
       <c r="H97" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I97" s="5" t="inlineStr">
@@ -7234,7 +6954,7 @@
       </c>
       <c r="H98" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I98" s="3" t="inlineStr">
@@ -7292,7 +7012,7 @@
       </c>
       <c r="H99" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I99" s="5" t="inlineStr">
@@ -7350,7 +7070,7 @@
       </c>
       <c r="H100" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I100" s="3" t="inlineStr">
@@ -7408,7 +7128,7 @@
       </c>
       <c r="H101" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I101" s="5" t="inlineStr">
@@ -7466,7 +7186,7 @@
       </c>
       <c r="H102" s="3" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I102" s="3" t="inlineStr">
@@ -7524,7 +7244,7 @@
       </c>
       <c r="H103" s="5" t="inlineStr">
         <is>
-          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+          <t>ERROR: Connection error caused by: ConnectionError(Connection error caused by: NewConnectionError(HTTPConnection(host='localhost', port=9200): Failed to establish a new connection: [WinError 10061] No connection could be made because the target machine actively refused it))</t>
         </is>
       </c>
       <c r="I103" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P10: GitHub push prep — eval results, SETUP.md, .gitignore cleanup
- README: fill evaluation results (Recall@8 80%, MRR 72%, Citation 52%,
  Faithfulness 19.5%, Refusal 4%) from 25-query checkpoint
- Add SETUP.md quick-start guide (docker-compose → pip → .env → ingest → run)
- .env.example: expand to full 4-key schema + all model/retrieval vars
- .gitignore: add ui/.next/, reports/eval_checkpoint.json,
  reports/evaluation_results.json, .venv, Jupyter, IDE dirs
- Untrack runtime report files (eval_checkpoint, evaluation_results)
- api/main.py: CORS extended to 127.0.0.1 variants (ports 3000 + 3001)
- Add demo.png UI screenshot referenced by README

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/evaluation_report.xlsx
+++ b/reports/evaluation_report.xlsx
@@ -1264,7 +1264,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Small (0.2-0.5)</t>
+          <t>Small Effect (0.2 - 0.5)</t>
         </is>
       </c>
     </row>
@@ -1300,14 +1300,14 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Large (&gt;=0.8)</t>
+          <t>Large Effect (&gt;= 0.8)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Factual vs Multi hop</t>
+          <t>Factual vs Multi_hop</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -1336,14 +1336,14 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Large (&gt;=0.8)</t>
+          <t>Large Effect (&gt;= 0.8)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Factual vs Multi hop</t>
+          <t>Factual vs Multi_hop</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -1372,14 +1372,14 @@
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Large (&gt;=0.8)</t>
+          <t>Large Effect (&gt;= 0.8)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Interpretive vs Multi hop</t>
+          <t>Interpretive vs Multi_hop</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -1408,14 +1408,14 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Large (&gt;=0.8)</t>
+          <t>Large Effect (&gt;= 0.8)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Interpretive vs Multi hop</t>
+          <t>Interpretive vs Multi_hop</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -1444,7 +1444,7 @@
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Negligible (&lt;0.2)</t>
+          <t>Negligible (&lt; 0.2)</t>
         </is>
       </c>
     </row>
@@ -1459,7 +1459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N28"/>
+  <dimension ref="A1:N103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3198,6 +3198,4356 @@
         <v>0</v>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Q026</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>pov</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>How does the estimated coefficient on wealth affect bequests according to the report on page 17 of the Gao Report: 05 Smallbiz?</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr"/>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>pov_gao_05_smallbiz, p.17</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J29" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Q027</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>multi_hop</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>judgment</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>What is the significance of Congress' failure to act on the IRS rulings of 1970 and 1971, and how does this relate to the concept of legislative acquiescence in the context of § 170 and § 501(c)(3)?</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr"/>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>judgment_07_bob_jones_university_v_united_states, p.12</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J30" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Q028</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>interpretive</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>act</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>How does the definition of 'receipt' in IRC §61 impact the tax treatment of a qualified taxpayer who has a right to receive, but has not yet actually received, an agricultural commodity under a 1983 payment-in-kind program?</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr"/>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>act_sec61, p.2</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J31" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K31" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Q029</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>act</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>What is the title of the section on page 3 of the provided document?</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr"/>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>act_sec212, p.3</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J32" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N32" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Q030</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>unanswerable</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>pov</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>What are the specific charitable donation limits for individuals under section 451(c) of the tax code?</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr"/>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>pov_tf_04_charitable, p.11</t>
+        </is>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J33" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Q031</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>unanswerable</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>judgment</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>What specific tax implications arose from the hedging transactions in the subsequent years following the Corn Products Refining Co. v. Commissioner case?</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr"/>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>judgment_19_arkansas_best_corporation_v_commissioner, p.5</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J34" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Q032</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>unanswerable</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>pov</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>What are the specific depreciation methods allowed for rental real estate enterprises under section 199A?</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr"/>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>pov_crs_08_qbi, p.6</t>
+        </is>
+      </c>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J35" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N35" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Q033</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>interpretive</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>judgment</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>How did the court in Old Colony Trust Co. v. Commissioner determine the measure of the benefit resulting to the beneficiary from coming into possession or enjoyment of the property after the expiration of a life estate?</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr"/>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>judgment_02_old_colony_trust_co_v_commissioner, p.5</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J36" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Q034</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>pov</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>What variables are included in Xi?</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr"/>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>pov_gao_04_penalties, p.10</t>
+        </is>
+      </c>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J37" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N37" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Q035</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>unanswerable</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>judgment</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>What is the specific procedure for filing an amended tax return in cases where the taxpayer has claimed a loss on a mortgaged property?</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr"/>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>judgment_15_crane_v_commissioner, p.6</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J38" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L38" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N38" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Q036</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>multi_hop</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>judgment</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>What is the interpretation of the term 'gift' in the context of the gift tax statute, and how does this interpretation relate to the treatment of transfers made for consideration, as discussed in the context of estate tax and income tax?</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr"/>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>judgment_13_faridessultaneh_v_commissioner, p.4</t>
+        </is>
+      </c>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I39" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J39" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L39" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N39" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Q037</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>pov</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>What does gross income include under section 61 of the Code?</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr"/>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>pov_jct_06_capgains, p.4</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J40" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L40" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N40" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Q038</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>interpretive</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>pov</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>How does the introduction of the concept of a 'consolidated reporting statement' in section 6045(b) impact the deadline for reporting entities to furnish required payee statements, and what implications does this have for the penalty imposed by section 6722?</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr"/>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>pov_crs_12_hobby_loss, p.2</t>
+        </is>
+      </c>
+      <c r="H41" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I41" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J41" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L41" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N41" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Q039</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>act</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>On what date was Pub. L. 97–248 enacted?</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr"/>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>act_sec163, p.11</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J42" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L42" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N42" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Q040</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>unanswerable</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>pov</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>What is the specific procedure for claiming the Mortgage Interest Deduction on a tax return for a primary residence in a different country?</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr"/>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>pov_gao_01_tax_exempt, p.27</t>
+        </is>
+      </c>
+      <c r="H43" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I43" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J43" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K43" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L43" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M43" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N43" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>Q041</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>interpretive</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>pov</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>How do the proposed regulations under section 1446(f) balance the need to reduce overwithholding with the requirement to verify the accuracy of certifications, particularly in cases where certifications are received after the date of payment?</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr"/>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>pov_crs_06_capital_gains, p.5</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J44" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K44" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L44" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M44" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N44" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Q042</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>multi_hop</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>judgment</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>What are the two elements that comprise the sales price as of January 15, 1979, and how do these elements relate to the partnership's obligation to pay the sales price of $1,224,000 as stated in the sales agreement?</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr"/>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>judgment_21_estate_of_franklin_v_commissioner, p.9</t>
+        </is>
+      </c>
+      <c r="H45" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I45" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J45" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K45" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M45" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N45" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Q043</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>act</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>What is the applicable amount for a joint return or a surviving spouse under IRC §68?</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr"/>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>act_sec68, p.2</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J46" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L46" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N46" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Q044</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>unanswerable</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>judgment</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>What is the specific procedure for filing an appeal in a case like United States v. Kirby Lumber Co.?</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr"/>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>judgment_12_united_states_v_kirby_lumber, p.1</t>
+        </is>
+      </c>
+      <c r="H47" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I47" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J47" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K47" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L47" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M47" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N47" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>Q045</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>interpretive</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>pov</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>How does the vehicle cents-per-mile valuation rule define 'personal miles' for purposes of calculating the value of the benefit provided to an employee, and what implications does this definition have for the application of the rule?</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr"/>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>pov_jct_07_penalties, p.6</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I48" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J48" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K48" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L48" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M48" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N48" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Q046</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>unanswerable</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>tax</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>What is the deadline for filing an amended return for social security benefits received in 2024?</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr"/>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>tax_pub17, p.66</t>
+        </is>
+      </c>
+      <c r="H49" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I49" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J49" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K49" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L49" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M49" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N49" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>Q047</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>judgment</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>What is compared to the good will of an old partnership in the context of expenses?</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr"/>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>judgment_04_welch_v_helvering, p.3</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I50" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J50" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K50" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L50" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M50" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N50" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Q048</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>tax</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>What type of businesses does this chapter not apply to?</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr"/>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>tax_pub334, p.28</t>
+        </is>
+      </c>
+      <c r="H51" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I51" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J51" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K51" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L51" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M51" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N51" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>Q049</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>tax</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>What conditions must an eating facility meet to be considered an employer-operated eating facility for employees?</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr"/>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>tax_pub15b, p.19</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I52" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J52" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K52" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L52" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M52" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N52" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Q050</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>multi_hop</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>pov</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>What is the impact of including stock option income on NIPA Wages and Salaries, and how does this compare to the effect of spread income deductions on NIPA Profits Before Tax?</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr"/>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
+          <t>pov_gao_02_likekind, p.18</t>
+        </is>
+      </c>
+      <c r="H53" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I53" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J53" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K53" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L53" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M53" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N53" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>Q051</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>interpretive</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>act</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>How does the context of corporate reorganizations under IRC §368 inform the interpretation of a 'reorganization' for tax purposes?</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr"/>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>act_sec368, p.3</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I54" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J54" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K54" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L54" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M54" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N54" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Q052</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>judgment</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>On what grounds did respondent disallow petitioners' management fees deduction?</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr"/>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>judgment_20_grodt_mckay_realty_v_commissioner, p.11</t>
+        </is>
+      </c>
+      <c r="H55" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I55" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J55" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L55" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N55" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>Q053</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>interpretive</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>act</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>How does the term 'applicable policyholder' expand to include related persons under IRC §101, and what are the implications of this expansion for employer-owned life insurance contracts?</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr"/>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>act_sec101, p.5</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I56" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J56" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L56" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N56" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>Q054</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>pov</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>What is the adjusted gross income limitation under section 25B(b)(1)(A) for determining the retirement savings contributions credit for married taxpayers filing a joint return in 2024?</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr"/>
+      <c r="G57" s="5" t="inlineStr">
+        <is>
+          <t>pov_crs_03_charitable, p.3</t>
+        </is>
+      </c>
+      <c r="H57" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I57" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J57" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K57" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L57" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M57" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N57" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>Q055</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>interpretive</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>tax</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>How does the distinction between 'property held for personal use' and 'property used for the production of income' impact the tax treatment of gains and losses from the sale or exchange of such properties?</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr"/>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>tax_pub544, p.30</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I58" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J58" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K58" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L58" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M58" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N58" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>Q056</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>multi_hop</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>judgment</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>What is the purpose of the section regarding corporate reorganizations, and how does this purpose relate to the underlying presupposition that the readjustment shall be undertaken for reasons germane to the conduct of the venture in hand?</t>
+        </is>
+      </c>
+      <c r="F59" s="5" t="inlineStr"/>
+      <c r="G59" s="5" t="inlineStr">
+        <is>
+          <t>judgment_08_gregory_v_helvering, p.3</t>
+        </is>
+      </c>
+      <c r="H59" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I59" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J59" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K59" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L59" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M59" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N59" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>Q057</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>judgment</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>What is the age limit for the protected class under the ADEA, as stated in § 631(a)?</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr"/>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t>judgment_27_textron_inc_v_united_states, p.15</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I60" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J60" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K60" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L60" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M60" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N60" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>Q058</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>act</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>What was the substitution made by Pub. L. 101–508, § 11101(d)(1)(F) in Subsec. (d)(3)(B) of IRC § 151?</t>
+        </is>
+      </c>
+      <c r="F61" s="5" t="inlineStr"/>
+      <c r="G61" s="5" t="inlineStr">
+        <is>
+          <t>act_sec151, p.3</t>
+        </is>
+      </c>
+      <c r="H61" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I61" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J61" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K61" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L61" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M61" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N61" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>Q059</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>multi_hop</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>tax</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>What is the business-use requirement for listed property, and how does this requirement relate to claiming a special depreciation allowance or the section 179 deduction?</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr"/>
+      <c r="G62" s="3" t="inlineStr">
+        <is>
+          <t>tax_pub946, p.51</t>
+        </is>
+      </c>
+      <c r="H62" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I62" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J62" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K62" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L62" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M62" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N62" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>Q060</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>interpretive</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>judgment</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>How did the court distinguish between an investor and a trader in the securities market, and what implications does this distinction have for the plaintiffs' activities?</t>
+        </is>
+      </c>
+      <c r="F63" s="5" t="inlineStr"/>
+      <c r="G63" s="5" t="inlineStr">
+        <is>
+          <t>judgment_26_moller_v_united_states, p.6</t>
+        </is>
+      </c>
+      <c r="H63" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I63" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J63" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K63" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L63" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M63" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N63" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>Q061</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>pov</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>What is the basis of the property received in a like-kind exchange of real property?</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr"/>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>pov_jct_01_tcja, p.12</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I64" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J64" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K64" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L64" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M64" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N64" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>Q062</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>multi_hop</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>judgment</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>What is the significance of the phrase 'gains or profits and income derived from any source whatever' in § 22 (a), and how does the court's interpretation of this phrase relate to the characterization of income in Eisner v. Macomber?</t>
+        </is>
+      </c>
+      <c r="F65" s="5" t="inlineStr"/>
+      <c r="G65" s="5" t="inlineStr">
+        <is>
+          <t>judgment_01_commissioner_v_glenshaw_glass, p.3</t>
+        </is>
+      </c>
+      <c r="H65" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I65" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J65" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K65" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L65" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M65" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N65" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>Q063</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>pov</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>In the case of Edem v. Comm’r, T.C. Memo. 2013-238, what was the result of the taxpayers' failure to introduce evidence to substantiate business expenses?</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr"/>
+      <c r="G66" s="3" t="inlineStr">
+        <is>
+          <t>pov_irs_01_sec162, p.5</t>
+        </is>
+      </c>
+      <c r="H66" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I66" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J66" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K66" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L66" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M66" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N66" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>Q064</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>multi_hop</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>act</t>
+        </is>
+      </c>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>What is the definition of a 'tax-exempt obligation' under IRC §265, and how does this definition relate to the concept of 'interest' as described in the same section?</t>
+        </is>
+      </c>
+      <c r="F67" s="5" t="inlineStr"/>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>act_sec265, p.4</t>
+        </is>
+      </c>
+      <c r="H67" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I67" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J67" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K67" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L67" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M67" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N67" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>Q065</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>interpretive</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>act</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>How does the treatment of a gift, bequest, devise, or inheritance of income from property, as outlined in IRC §102, impact the gross income of a beneficiary under subchapter J, particularly when the payment is made at intervals?</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr"/>
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t>act_sec102, p.1</t>
+        </is>
+      </c>
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I68" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J68" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K68" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L68" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M68" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N68" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t>Q066</t>
+        </is>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>act</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E69" s="5" t="inlineStr">
+        <is>
+          <t>What year was subsection (e) added to IRC §263?</t>
+        </is>
+      </c>
+      <c r="F69" s="5" t="inlineStr"/>
+      <c r="G69" s="5" t="inlineStr">
+        <is>
+          <t>act_sec263, p.3</t>
+        </is>
+      </c>
+      <c r="H69" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I69" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J69" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K69" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L69" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M69" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N69" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>Q067</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>multi_hop</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>act</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>What is the definition of a capital asset under IRC §1221, and how does this definition impact the categorization of assets under the provided legal text on page 3?</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr"/>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>act_sec1221, p.3</t>
+        </is>
+      </c>
+      <c r="H70" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I70" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J70" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K70" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L70" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M70" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N70" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="inlineStr">
+        <is>
+          <t>Q068</t>
+        </is>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>multi_hop</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>act</t>
+        </is>
+      </c>
+      <c r="D71" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E71" s="5" t="inlineStr">
+        <is>
+          <t>What is the definition of taxable income for corporations prior to amendment, and how does this compare to the definition for individuals who do not itemize their deductions as stated in subsection (b) after the amendment?</t>
+        </is>
+      </c>
+      <c r="F71" s="5" t="inlineStr"/>
+      <c r="G71" s="5" t="inlineStr">
+        <is>
+          <t>act_sec63, p.3</t>
+        </is>
+      </c>
+      <c r="H71" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I71" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J71" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K71" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L71" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M71" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N71" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>Q069</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>pov</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>What position does the taxpayer take regarding the basis of USP in the FP nonqualified preferred stock?</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="inlineStr"/>
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>pov_crs_11_reorg, p.12</t>
+        </is>
+      </c>
+      <c r="H72" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I72" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J72" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K72" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L72" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M72" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N72" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>Q070</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>pov</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>According to the IRS press release IR-2002-05, what was one purpose for the National Research Program?</t>
+        </is>
+      </c>
+      <c r="F73" s="5" t="inlineStr"/>
+      <c r="G73" s="5" t="inlineStr">
+        <is>
+          <t>pov_gao_03_retirement, p.21</t>
+        </is>
+      </c>
+      <c r="H73" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I73" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J73" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K73" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L73" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M73" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N73" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>Q071</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>pov</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>What is the adjusted gross income limitation under section 25B(b)(1)(A) for determining the retirement savings contributions credit for married taxpayers filing a joint return in 2023?</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="inlineStr"/>
+      <c r="G74" s="3" t="inlineStr">
+        <is>
+          <t>pov_crs_07_ira, p.3</t>
+        </is>
+      </c>
+      <c r="H74" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I74" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J74" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K74" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L74" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M74" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N74" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t>Q072</t>
+        </is>
+      </c>
+      <c r="B75" s="5" t="inlineStr">
+        <is>
+          <t>unanswerable</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>act</t>
+        </is>
+      </c>
+      <c r="D75" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E75" s="5" t="inlineStr">
+        <is>
+          <t>What is the specific procedure for filing an amended tax return for a like-kind exchange under IRC Section 1031?</t>
+        </is>
+      </c>
+      <c r="F75" s="5" t="inlineStr"/>
+      <c r="G75" s="5" t="inlineStr">
+        <is>
+          <t>act_sec1031, p.3</t>
+        </is>
+      </c>
+      <c r="H75" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I75" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J75" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K75" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L75" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M75" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N75" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>Q073</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>judgment</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>What is the predecessor of Section 61(a) in the 1954 Code?</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="inlineStr"/>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>judgment_03_cesarini_v_united_states, p.4</t>
+        </is>
+      </c>
+      <c r="H76" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I76" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J76" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K76" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L76" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M76" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N76" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="5" t="inlineStr">
+        <is>
+          <t>Q074</t>
+        </is>
+      </c>
+      <c r="B77" s="5" t="inlineStr">
+        <is>
+          <t>unanswerable</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>tax</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E77" s="5" t="inlineStr">
+        <is>
+          <t>What are the specific filing requirements for charitable contributions made to foreign organizations?</t>
+        </is>
+      </c>
+      <c r="F77" s="5" t="inlineStr"/>
+      <c r="G77" s="5" t="inlineStr">
+        <is>
+          <t>tax_pub526, p.21</t>
+        </is>
+      </c>
+      <c r="H77" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I77" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J77" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K77" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L77" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M77" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N77" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>Q075</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>judgment</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>What is the test of nondeductibility according to Tank Truck Rentals v. Commissioner?</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr"/>
+      <c r="G78" s="3" t="inlineStr">
+        <is>
+          <t>judgment_05_commissioner_v_tellier, p.4</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I78" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J78" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K78" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L78" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M78" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N78" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="5" t="inlineStr">
+        <is>
+          <t>Q076</t>
+        </is>
+      </c>
+      <c r="B79" s="5" t="inlineStr">
+        <is>
+          <t>interpretive</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>pov</t>
+        </is>
+      </c>
+      <c r="D79" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E79" s="5" t="inlineStr">
+        <is>
+          <t>How do the Treasury Department and the IRS expect comments to address the potential applicability of state charity laws to charitable LLCs, in terms of ensuring that assets remain dedicated to an exempt purpose and preventing private inurement?</t>
+        </is>
+      </c>
+      <c r="F79" s="5" t="inlineStr"/>
+      <c r="G79" s="5" t="inlineStr">
+        <is>
+          <t>pov_crs_04_exempt_orgs, p.8</t>
+        </is>
+      </c>
+      <c r="H79" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I79" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J79" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K79" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L79" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M79" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N79" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>Q077</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>pov</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>What is the purpose of Section 111 of the Code as described in the provided text?</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="inlineStr"/>
+      <c r="G80" s="3" t="inlineStr">
+        <is>
+          <t>pov_crs_01_gross_income, p.4</t>
+        </is>
+      </c>
+      <c r="H80" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I80" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J80" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K80" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L80" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M80" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N80" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="5" t="inlineStr">
+        <is>
+          <t>Q078</t>
+        </is>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>pov</t>
+        </is>
+      </c>
+      <c r="D81" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E81" s="5" t="inlineStr">
+        <is>
+          <t>What is the threshold for a corporation to obtain a qualified appraisal for deductions of property claimed?</t>
+        </is>
+      </c>
+      <c r="F81" s="5" t="inlineStr"/>
+      <c r="G81" s="5" t="inlineStr">
+        <is>
+          <t>pov_tf_03_corporate, p.13</t>
+        </is>
+      </c>
+      <c r="H81" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I81" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J81" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K81" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L81" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M81" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N81" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>Q079</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>pov</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t>What is the default classification for a domestic eligible entity with two or more owners under § 301.7701-3(b)(1)?</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="inlineStr"/>
+      <c r="G82" s="3" t="inlineStr">
+        <is>
+          <t>pov_crs_05_like_kind, p.8</t>
+        </is>
+      </c>
+      <c r="H82" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I82" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J82" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K82" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L82" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M82" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N82" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="5" t="inlineStr">
+        <is>
+          <t>Q080</t>
+        </is>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>judgment</t>
+        </is>
+      </c>
+      <c r="D83" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E83" s="5" t="inlineStr">
+        <is>
+          <t>In what year was the case of United States v. Ross decided?</t>
+        </is>
+      </c>
+      <c r="F83" s="5" t="inlineStr"/>
+      <c r="G83" s="5" t="inlineStr">
+        <is>
+          <t>judgment_23_commissioner_v_flowers, p.11</t>
+        </is>
+      </c>
+      <c r="H83" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I83" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J83" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K83" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L83" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M83" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N83" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>Q081</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>interpretive</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>act</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E84" s="3" t="inlineStr">
+        <is>
+          <t>How does the statutory period for assessing a deficiency attributable to an activity, as outlined in IRC §183, interact with the general provisions of law or rules of law that would otherwise prevent such an assessment, particularly in cases where a taxpayer has made an election under paragraph (1) with respect to that activity?</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="inlineStr"/>
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>act_sec183, p.2</t>
+        </is>
+      </c>
+      <c r="H84" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I84" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J84" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K84" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L84" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M84" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N84" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="5" t="inlineStr">
+        <is>
+          <t>Q082</t>
+        </is>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>interpretive</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="inlineStr">
+        <is>
+          <t>judgment</t>
+        </is>
+      </c>
+      <c r="D85" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E85" s="5" t="inlineStr">
+        <is>
+          <t>How did the court in Cheek v. United States interpret the willfulness requirement in the context of a defendant's good faith belief about the constitutionality of the income tax law as applied to them?</t>
+        </is>
+      </c>
+      <c r="F85" s="5" t="inlineStr"/>
+      <c r="G85" s="5" t="inlineStr">
+        <is>
+          <t>judgment_11_cheek_v_united_states, p.8</t>
+        </is>
+      </c>
+      <c r="H85" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I85" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J85" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K85" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L85" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M85" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N85" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>Q083</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>interpretive</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>act</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="inlineStr">
+        <is>
+          <t>What implications does the transfer to a controlled corporation under IRC §351 have on the tax treatment of the transferor's assets, and how does this provision balance the interests of the transferor and the controlled corporation?</t>
+        </is>
+      </c>
+      <c r="F86" s="3" t="inlineStr"/>
+      <c r="G86" s="3" t="inlineStr">
+        <is>
+          <t>act_sec351, p.3</t>
+        </is>
+      </c>
+      <c r="H86" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I86" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J86" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K86" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L86" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M86" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N86" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="5" t="inlineStr">
+        <is>
+          <t>Q084</t>
+        </is>
+      </c>
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>interpretive</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="inlineStr">
+        <is>
+          <t>judgment</t>
+        </is>
+      </c>
+      <c r="D87" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E87" s="5" t="inlineStr">
+        <is>
+          <t>How does the Board distinguish between 'allowances' and 'compensation' in the context of determining taxable income, as evident from the decisions cited in the case?</t>
+        </is>
+      </c>
+      <c r="F87" s="5" t="inlineStr"/>
+      <c r="G87" s="5" t="inlineStr">
+        <is>
+          <t>judgment_25_benaglia_v_commissioner, p.2</t>
+        </is>
+      </c>
+      <c r="H87" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I87" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J87" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K87" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L87" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M87" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N87" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t>Q085</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>multi_hop</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>pov</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E88" s="3" t="inlineStr">
+        <is>
+          <t>How does the limitation on the exclusion under § 121 due to prior depreciation deductions relate to the deductibility of losses under § 165, particularly for losses of property not connected with a trade or business?</t>
+        </is>
+      </c>
+      <c r="F88" s="3" t="inlineStr"/>
+      <c r="G88" s="3" t="inlineStr">
+        <is>
+          <t>pov_crs_02_business_expense, p.9</t>
+        </is>
+      </c>
+      <c r="H88" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I88" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J88" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K88" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L88" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M88" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N88" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="5" t="inlineStr">
+        <is>
+          <t>Q086</t>
+        </is>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
+        <is>
+          <t>interpretive</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>judgment</t>
+        </is>
+      </c>
+      <c r="D89" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E89" s="5" t="inlineStr">
+        <is>
+          <t>How does the court's interpretation of the Fifth Amendment's protection against self-incrimination relate to the government's role in upholding the law, as discussed in the context of Olmstead v. United States?</t>
+        </is>
+      </c>
+      <c r="F89" s="5" t="inlineStr"/>
+      <c r="G89" s="5" t="inlineStr">
+        <is>
+          <t>judgment_29_davis_v_united_states, p.21</t>
+        </is>
+      </c>
+      <c r="H89" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I89" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J89" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K89" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L89" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M89" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N89" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>Q087</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>pov</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E90" s="3" t="inlineStr">
+        <is>
+          <t>For tax years beginning after 2017, how long do you have to complete the rollover of a qualified plan loan offset?</t>
+        </is>
+      </c>
+      <c r="F90" s="3" t="inlineStr"/>
+      <c r="G90" s="3" t="inlineStr">
+        <is>
+          <t>pov_jct_03_charitable, p.23</t>
+        </is>
+      </c>
+      <c r="H90" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I90" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J90" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K90" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L90" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M90" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N90" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="5" t="inlineStr">
+        <is>
+          <t>Q088</t>
+        </is>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C91" s="5" t="inlineStr">
+        <is>
+          <t>pov</t>
+        </is>
+      </c>
+      <c r="D91" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E91" s="5" t="inlineStr">
+        <is>
+          <t>What is the amount excludable from an employee's gross income for qualified adoption expenses furnished pursuant to an adoption assistance program, and at what modified adjusted gross income level does it begin to phase out?</t>
+        </is>
+      </c>
+      <c r="F91" s="5" t="inlineStr"/>
+      <c r="G91" s="5" t="inlineStr">
+        <is>
+          <t>pov_jct_04_retirement, p.15</t>
+        </is>
+      </c>
+      <c r="H91" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I91" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J91" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K91" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L91" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M91" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N91" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>Q089</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>multi_hop</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>tax</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E92" s="3" t="inlineStr">
+        <is>
+          <t>How is the unadjusted basis of a car determined for depreciation deduction purposes, and what happens to the unrecovered basis after the recovery period ends?</t>
+        </is>
+      </c>
+      <c r="F92" s="3" t="inlineStr"/>
+      <c r="G92" s="3" t="inlineStr">
+        <is>
+          <t>tax_pub463, p.30</t>
+        </is>
+      </c>
+      <c r="H92" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I92" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J92" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K92" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L92" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M92" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N92" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="5" t="inlineStr">
+        <is>
+          <t>Q090</t>
+        </is>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>interpretive</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>tax</t>
+        </is>
+      </c>
+      <c r="D93" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E93" s="5" t="inlineStr">
+        <is>
+          <t>How do the rules for amortizing business startup and organizational costs differ for costs paid or incurred before October 23, 2004, versus those paid or incurred on or after this date, and what implications does this have for the treatment of these costs under the tax law?</t>
+        </is>
+      </c>
+      <c r="F93" s="5" t="inlineStr"/>
+      <c r="G93" s="5" t="inlineStr">
+        <is>
+          <t>tax_pub535, p.29</t>
+        </is>
+      </c>
+      <c r="H93" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I93" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J93" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K93" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L93" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M93" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N93" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>Q091</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>pov</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>What forms can separable activities take, according to the provided text?</t>
+        </is>
+      </c>
+      <c r="F94" s="3" t="inlineStr"/>
+      <c r="G94" s="3" t="inlineStr">
+        <is>
+          <t>pov_crs_10_penalties, p.4</t>
+        </is>
+      </c>
+      <c r="H94" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I94" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J94" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K94" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L94" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M94" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N94" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="5" t="inlineStr">
+        <is>
+          <t>Q092</t>
+        </is>
+      </c>
+      <c r="B95" s="5" t="inlineStr">
+        <is>
+          <t>interpretive</t>
+        </is>
+      </c>
+      <c r="C95" s="5" t="inlineStr">
+        <is>
+          <t>act</t>
+        </is>
+      </c>
+      <c r="D95" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E95" s="5" t="inlineStr">
+        <is>
+          <t>What is the implication of the 1976 amendment to subsection (c) of IRC §1001, which substituted the provision recognizing the entire amount of gain or loss, and how does it affect the determination of gain or loss to be recognized?</t>
+        </is>
+      </c>
+      <c r="F95" s="5" t="inlineStr"/>
+      <c r="G95" s="5" t="inlineStr">
+        <is>
+          <t>act_sec1001, p.2</t>
+        </is>
+      </c>
+      <c r="H95" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I95" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J95" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K95" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L95" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M95" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N95" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>Q093</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>multi_hop</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>act</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>What is the definition of personal property under the former subsection (f), and how does the redesignation of subsections by Pub. L. 101–508 affect the computation of the allowance under subsection (a) with respect to such property?</t>
+        </is>
+      </c>
+      <c r="F96" s="3" t="inlineStr"/>
+      <c r="G96" s="3" t="inlineStr">
+        <is>
+          <t>act_sec167, p.6</t>
+        </is>
+      </c>
+      <c r="H96" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I96" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J96" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K96" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L96" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M96" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N96" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="5" t="inlineStr">
+        <is>
+          <t>Q094</t>
+        </is>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
+        <is>
+          <t>interpretive</t>
+        </is>
+      </c>
+      <c r="C97" s="5" t="inlineStr">
+        <is>
+          <t>judgment</t>
+        </is>
+      </c>
+      <c r="D97" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E97" s="5" t="inlineStr">
+        <is>
+          <t>How did the court interpret the application of § 752(c) in relation to § 752(a) and (b) transactions, and what was the underlying rationale for this interpretation?</t>
+        </is>
+      </c>
+      <c r="F97" s="5" t="inlineStr"/>
+      <c r="G97" s="5" t="inlineStr">
+        <is>
+          <t>judgment_16_commissioner_v_tufts, p.9</t>
+        </is>
+      </c>
+      <c r="H97" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I97" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J97" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K97" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L97" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M97" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N97" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t>Q095</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>judgment</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="inlineStr">
+        <is>
+          <t>What sections give non-recognition treatment to sales and reinvestment transactions in limited circumstances?</t>
+        </is>
+      </c>
+      <c r="F98" s="3" t="inlineStr"/>
+      <c r="G98" s="3" t="inlineStr">
+        <is>
+          <t>judgment_10_starker_v_united_states, p.4</t>
+        </is>
+      </c>
+      <c r="H98" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I98" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J98" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K98" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L98" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M98" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N98" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="5" t="inlineStr">
+        <is>
+          <t>Q096</t>
+        </is>
+      </c>
+      <c r="B99" s="5" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C99" s="5" t="inlineStr">
+        <is>
+          <t>judgment</t>
+        </is>
+      </c>
+      <c r="D99" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E99" s="5" t="inlineStr">
+        <is>
+          <t>In what year was the Eisner v. Macomber case decided?</t>
+        </is>
+      </c>
+      <c r="F99" s="5" t="inlineStr"/>
+      <c r="G99" s="5" t="inlineStr">
+        <is>
+          <t>judgment_09_cottage_savings_association_v_commissioner, p.6</t>
+        </is>
+      </c>
+      <c r="H99" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I99" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J99" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K99" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L99" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M99" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N99" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="3" t="inlineStr">
+        <is>
+          <t>Q097</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>multi_hop</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>act</t>
+        </is>
+      </c>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E100" s="3" t="inlineStr">
+        <is>
+          <t>What requirements must an organization meet to limit charges for emergency or medically necessary care, and how do these requirements relate to the billing and collection actions described in paragraph (6)?</t>
+        </is>
+      </c>
+      <c r="F100" s="3" t="inlineStr"/>
+      <c r="G100" s="3" t="inlineStr">
+        <is>
+          <t>act_sec501, p.15</t>
+        </is>
+      </c>
+      <c r="H100" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I100" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J100" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K100" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L100" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M100" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N100" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="5" t="inlineStr">
+        <is>
+          <t>Q098</t>
+        </is>
+      </c>
+      <c r="B101" s="5" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>act</t>
+        </is>
+      </c>
+      <c r="D101" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E101" s="5" t="inlineStr">
+        <is>
+          <t>What requirements must a pension plan satisfy under IRC §401(a) to qualify as tax-exempt?</t>
+        </is>
+      </c>
+      <c r="F101" s="5" t="inlineStr"/>
+      <c r="G101" s="5" t="inlineStr">
+        <is>
+          <t>act_sec401, p.1</t>
+        </is>
+      </c>
+      <c r="H101" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I101" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J101" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K101" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L101" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M101" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N101" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>Q099</t>
+        </is>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>multi_hop</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>act</t>
+        </is>
+      </c>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E102" s="3" t="inlineStr">
+        <is>
+          <t>What is the treatment of charitable contributions made to organizations described in section 170(b)(1)(A), and how does this treatment relate to the rules regarding donor advised funds as defined in section 4966(d)(2)?</t>
+        </is>
+      </c>
+      <c r="F102" s="3" t="inlineStr"/>
+      <c r="G102" s="3" t="inlineStr">
+        <is>
+          <t>act_sec170, p.20</t>
+        </is>
+      </c>
+      <c r="H102" s="3" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I102" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J102" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K102" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L102" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M102" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N102" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="5" t="inlineStr">
+        <is>
+          <t>Q100</t>
+        </is>
+      </c>
+      <c r="B103" s="5" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>tax</t>
+        </is>
+      </c>
+      <c r="D103" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E103" s="5" t="inlineStr">
+        <is>
+          <t>How is the fair market value of digital assets determined when received as payment for services?</t>
+        </is>
+      </c>
+      <c r="F103" s="5" t="inlineStr"/>
+      <c r="G103" s="5" t="inlineStr">
+        <is>
+          <t>tax_pub550, p.59</t>
+        </is>
+      </c>
+      <c r="H103" s="5" t="inlineStr">
+        <is>
+          <t>ERROR: BadRequestError(400, 'media_type_header_exception', 'Invalid media-type value on headers [Accept, Content-Type]', Accept version must be either version 8 or 7, but found 9. Accept=application/vnd.elasticsearch+json; compatible-with=9)</t>
+        </is>
+      </c>
+      <c r="I103" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J103" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K103" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L103" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M103" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N103" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>